<commit_message>
fix: align request scope and private report provenance
</commit_message>
<xml_diff>
--- a/docs/evidence/direction-report-redesign/synthetic-populated-report.xlsx
+++ b/docs/evidence/direction-report-redesign/synthetic-populated-report.xlsx
@@ -1265,7 +1265,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Gastos activos · base presupuestal del intervalo</t>
+          <t>Gastos activos · base fiscal canónica documental del intervalo</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -1615,7 +1615,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Gastos activos · base presupuestal del intervalo</t>
+          <t>Gastos activos · base fiscal canónica documental del intervalo</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">

</xml_diff>

<commit_message>
fix: bound tournament projections and require scope manifests
</commit_message>
<xml_diff>
--- a/docs/evidence/direction-report-redesign/synthetic-populated-report.xlsx
+++ b/docs/evidence/direction-report-redesign/synthetic-populated-report.xlsx
@@ -663,7 +663,7 @@
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Identificador de cifras: df368fcdea11792214655d11bc2dc6c82f55571a14ed2dd7121b6ba18b3eb752</t>
+          <t>Identificador de cifras: 7e94a0efeecca34c66bcd633604ef83bf6d8eea58007f8d7177f780dad19903a</t>
         </is>
       </c>
       <c r="B5" s="2" t="n"/>
@@ -1121,7 +1121,7 @@
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Lecturas secuenciales con cortes individuales. Proyección mecánica, sin causalidad acreditada. Pagado documental no equivale a salida de caja.</t>
+          <t>Lecturas independientes con cortes individuales. Proyección mecánica, sin causalidad acreditada. Pagado documental no equivale a salida de caja.</t>
         </is>
       </c>
       <c r="B28" s="2" t="n"/>

</xml_diff>

<commit_message>
fix: batch executive reads and page authorized catalogs in SQL
</commit_message>
<xml_diff>
--- a/docs/evidence/direction-report-redesign/synthetic-populated-report.xlsx
+++ b/docs/evidence/direction-report-redesign/synthetic-populated-report.xlsx
@@ -663,7 +663,7 @@
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Identificador de cifras: 7e94a0efeecca34c66bcd633604ef83bf6d8eea58007f8d7177f780dad19903a</t>
+          <t>Identificador de cifras: dca1b11a7b54826717003fb31b52631f0575c7b717e2620eccd592b66eb048a6</t>
         </is>
       </c>
       <c r="B5" s="2" t="n"/>
@@ -788,7 +788,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr"/>
     </row>
-    <row r="12" ht="55" customHeight="1">
+    <row r="12" ht="70" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Comprometido documental</t>
@@ -809,12 +809,12 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Importe pagable de solicitudes creadas en el intervalo; incluye pagadas/cerradas y reembolsos. No se suma al ejercido.</t>
+          <t>Importe pagable de solicitudes creadas en el intervalo, con su estado actual; incluye enviadas, liquidadas y reembolsos. No equivale a deuda pendiente ni se suma al ejercido.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr"/>
     </row>
-    <row r="13" ht="55" customHeight="1">
+    <row r="13" ht="70" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Pagado documental</t>
@@ -835,7 +835,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Importe pagable con estado/registro de pago, de solicitudes creadas en el intervalo; no es flujo por fecha efectiva ni caja.</t>
+          <t>Importe pagable de solicitudes creadas en el intervalo, con su estado/registro actual de pago; no acredita por sí solo una transferencia ni es flujo por fecha efectiva o caja.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr"/>
@@ -1285,7 +1285,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="70" customHeight="1">
+    <row r="4" ht="100" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Torneo sintético Norte</t>
@@ -1306,7 +1306,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Importe pagable de solicitudes creadas en el intervalo; incluye pagadas/cerradas y reembolsos. No se suma al ejercido.</t>
+          <t>Importe pagable de solicitudes creadas en el intervalo, con su estado actual; incluye enviadas, liquidadas y reembolsos. No equivale a deuda pendiente ni se suma al ejercido.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -1321,7 +1321,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="70" customHeight="1">
+    <row r="5" ht="100" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Torneo sintético Norte</t>
@@ -1342,7 +1342,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Importe pagable con estado/registro de pago, de solicitudes creadas en el intervalo; no es flujo por fecha efectiva ni caja.</t>
+          <t>Importe pagable de solicitudes creadas en el intervalo, con su estado/registro actual de pago; no acredita por sí solo una transferencia ni es flujo por fecha efectiva o caja.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -1635,7 +1635,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="70" customHeight="1">
+    <row r="14" ht="100" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Torneo sintético Sur</t>
@@ -1656,7 +1656,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Importe pagable de solicitudes creadas en el intervalo; incluye pagadas/cerradas y reembolsos. No se suma al ejercido.</t>
+          <t>Importe pagable de solicitudes creadas en el intervalo, con su estado actual; incluye enviadas, liquidadas y reembolsos. No equivale a deuda pendiente ni se suma al ejercido.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1671,7 +1671,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="70" customHeight="1">
+    <row r="15" ht="100" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
           <t>Torneo sintético Sur</t>
@@ -1692,7 +1692,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Importe pagable con estado/registro de pago, de solicitudes creadas en el intervalo; no es flujo por fecha efectiva ni caja.</t>
+          <t>Importe pagable de solicitudes creadas en el intervalo, con su estado/registro actual de pago; no acredita por sí solo una transferencia ni es flujo por fecha efectiva o caja.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">

</xml_diff>